<commit_message>
refactor: simplify pipeline into minimal data pipeline architecture
- Create modular src/ structure: ingestion, validation, processing, metrics
- Replace config.ini with clean config.py with constants
- Rewrite main.py as simple orchestrator (load → validate → process → metrics)
- Remove AI-generated code: logger.py, excessive docstrings, complex abstractions
- Simplify requirements.txt: pandas + openpyxl only
- Remove unused files: docs/, templates/, old scripts
- Keep functions minimal and readable
- Verify end-to-end pipeline runs successfully

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/output/West_Market_Summary.xlsx
+++ b/data/output/West_Market_Summary.xlsx
@@ -415,14 +415,6 @@
   </sheetPr>
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>